<commit_message>
W2 - design properties for installation sequencing constraints
minimum_spacing_to_fresh_element and
minimum_age_before_adjacent_installation, bound
//diggs:DesignConformanceCriterion/diggs:designProperty like the seven
entries already there.

These are the constraints that actually control installation effects on
fresh adjacent columns. They are requirements rather than an order, so they
are criterion-shaped (designProperty + operator + limit) and need no schema
at all - the same finding DE1 made, that a DesignConformanceCriterion IS the
gate. Stating them this way also makes them checkable rather than inert.

sequenceRule needed no dictionary: its vocabulary is a GML enumeration.

Append verified with zero deletions; only this workbook regenerated, so no
quote-escaping collateral.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1287,22 +1287,63 @@
         <f>IF(ISNA(VLOOKUP(B9,AssociatedElements!B$2:B2947,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="16" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="G9" s="9" t="n"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>minimum_spacing_to_fresh_element</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Minimum spacing to a fresh element</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>The minimum plan distance permitted between an element being installed and a previously installed element that has not yet reached the age or strength at which it is unaffected by the installation. Controls installation effects - ground displacement, vibration and fresh concrete disturbance - on neighbours placed shortly before. Stated as a length; where a specification expresses it as a multiple of element diameter, the limit is the product of that multiple and the design diameter.</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2">
         <f>IF(ISNA(VLOOKUP(B10,AssociatedElements!B$2:B2948,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="13" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="13" t="n"/>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>minimum_age_before_adjacent_installation</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Minimum age before adjacent installation</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>The minimum elapsed time between completing one element and beginning installation of an adjacent element, so that the earlier element has gained enough strength to be undisturbed. The time-based companion to minimum_spacing_to_fresh_element: a specification typically states one, the other, or both, and together they are what an installation sequence is designed to satisfy.</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F10" s="13" t="n"/>
-      <c r="G10" s="9" t="n"/>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2">
@@ -1780,14 +1821,32 @@
         <f>IF(ISNA(VLOOKUP(B9,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B9" s="2" t="n"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>minimum_spacing_to_fresh_element</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
         <f>IF(ISNA(VLOOKUP(B10,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B10" s="20" t="n"/>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>minimum_age_before_adjacent_installation</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11">

</xml_diff>

<commit_message>
D6 - penetration_rate and torque as design properties
Writing D6's motivating example - a drilling refusal criterion, "penetration
rate below X AND torque above Y" - surfaced that neither property had a
designProperty entry, though both exist as MEASURED properties in
mwd_properties.xml. So the canonical use case for the new
CompositeAcceptanceCriterion could not be stated with resolvable vocabulary.

Each is documented as the design-side counterpart of the mwd_properties
entry naming the same quantity as measured. Not invention: established DIGGS
concepts given a design-side home, the same move S27-S31 made for each new
procedure's results.

logicalOperator needed no dictionary - it is a closed enumeration in the
schema.

Append verified with zero deletions; only this workbook regenerated, so no
quote-escaping collateral.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/designProperty.xlsx
@@ -1350,24 +1350,64 @@
         <f>IF(ISNA(VLOOKUP(B11,AssociatedElements!B$2:B2949,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="14" t="n"/>
-      <c r="E11" s="13" t="n"/>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>penetration_rate</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Penetration rate</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>The rate at which the installation tool advances into the ground, as a design property a conformance criterion may govern. The design-side counterpart of mwd_properties.xml#penetration_rate, which names the same quantity as MEASURED during drilling; this entry names it as the subject of a requirement. Together with torque it is the pair a drilling refusal rule is normally written on, and such a rule is conjunctive - see diggs:CompositeAcceptanceCriterion.</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F11" s="13" t="n"/>
-      <c r="G11" s="9" t="n"/>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2">
         <f>IF(ISNA(VLOOKUP(B12,AssociatedElements!B$2:B2950,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B12" s="13" t="n"/>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="13" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>torque</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Torque</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>The rotational force applied to the installation tool, as a design property a conformance criterion may govern. The design-side counterpart of mwd_properties.xml#torque, which names the same quantity as MEASURED during drilling. Paired with penetration_rate in a refusal criterion: neither alone defines refusal, which is why the combination is stated as a diggs:CompositeAcceptanceCriterion rather than left implicit in two co-scoped criteria.</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F12" s="13" t="n"/>
-      <c r="G12" s="9" t="n"/>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2">
@@ -1853,14 +1893,32 @@
         <f>IF(ISNA(VLOOKUP(B11,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B11" s="20" t="n"/>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>penetration_rate</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
         <f>IF(ISNA(VLOOKUP(B12,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B12" s="20" t="n"/>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>torque</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>//diggs:DesignConformanceCriterion/diggs:designProperty</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13">

</xml_diff>